<commit_message>
spatial requirements and constraints
</commit_message>
<xml_diff>
--- a/Battery.xlsx
+++ b/Battery.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emirsener/Desktop/Campus-Application/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28ECCF1D-A560-8347-8686-6DB455B50CD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A177CE26-5252-0441-AF0E-F6AF223DF9ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15940" xr2:uid="{EDF38AB8-B67A-6545-84A8-C231FAB8949A}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="27">
   <si>
     <t>Metrics</t>
   </si>
@@ -116,6 +116,9 @@
   </si>
   <si>
     <t>0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0, 0</t>
+  </si>
+  <si>
+    <t>Spatial requirement</t>
   </si>
 </sst>
 </file>
@@ -475,7 +478,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5344E307-70EA-9749-BC3D-54A83804696F}">
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="25.6640625" bestFit="1" customWidth="1"/>
@@ -544,8 +547,7 @@
         <v>16</v>
       </c>
       <c r="B8">
-        <f>1/15</f>
-        <v>6.6666666666666666E-2</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
@@ -601,6 +603,14 @@
       </c>
       <c r="B14">
         <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>26</v>
+      </c>
+      <c r="B15">
+        <v>6.1000000000000004E-3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>